<commit_message>
FEMS hourly data (NM+AZ)
</commit_message>
<xml_diff>
--- a/data/fems_latest_wxMinMax.xlsx
+++ b/data/fems_latest_wxMinMax.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q158"/>
+  <dimension ref="A1:T158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,7 +499,22 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>peak_wind_gust_time</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>solar_radiation_max</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>daily_precipitation_total</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>snow_flag</t>
         </is>
       </c>
     </row>
@@ -528,7 +543,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -560,8 +575,17 @@
       <c r="P2" t="n">
         <v>16</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="n">
+        <v>962</v>
+      </c>
+      <c r="S2" t="n">
         <v>0</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -589,7 +613,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -621,8 +645,17 @@
       <c r="P3" t="n">
         <v>22</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="n">
+        <v>929</v>
+      </c>
+      <c r="S3" t="n">
         <v>0</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -650,7 +683,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -682,8 +715,17 @@
       <c r="P4" t="n">
         <v>21</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="n">
+        <v>814</v>
+      </c>
+      <c r="S4" t="n">
         <v>0</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -711,7 +753,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -743,8 +785,17 @@
       <c r="P5" t="n">
         <v>11</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="n">
+        <v>759</v>
+      </c>
+      <c r="S5" t="n">
         <v>0</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -772,7 +823,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -804,8 +855,17 @@
       <c r="P6" t="n">
         <v>25</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="n">
+        <v>891</v>
+      </c>
+      <c r="S6" t="n">
         <v>0</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -833,7 +893,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -865,8 +925,17 @@
       <c r="P7" t="n">
         <v>16</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="n">
+        <v>810</v>
+      </c>
+      <c r="S7" t="n">
         <v>0</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -894,7 +963,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -926,8 +995,17 @@
       <c r="P8" t="n">
         <v>23</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="n">
+        <v>979</v>
+      </c>
+      <c r="S8" t="n">
         <v>0</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -955,7 +1033,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -987,8 +1065,17 @@
       <c r="P9" t="n">
         <v>9</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="n">
+        <v>982</v>
+      </c>
+      <c r="S9" t="n">
         <v>0</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1016,7 +1103,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1048,8 +1135,17 @@
       <c r="P10" t="n">
         <v>17</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="n">
+        <v>909</v>
+      </c>
+      <c r="S10" t="n">
         <v>0</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1077,7 +1173,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1109,8 +1205,17 @@
       <c r="P11" t="n">
         <v>16</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="n">
+        <v>967</v>
+      </c>
+      <c r="S11" t="n">
         <v>0</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1138,7 +1243,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1170,8 +1275,17 @@
       <c r="P12" t="n">
         <v>13</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="n">
+        <v>871</v>
+      </c>
+      <c r="S12" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1199,7 +1313,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1231,8 +1345,17 @@
       <c r="P13" t="n">
         <v>21</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="n">
+        <v>945</v>
+      </c>
+      <c r="S13" t="n">
         <v>0</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1260,7 +1383,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1292,8 +1415,17 @@
       <c r="P14" t="n">
         <v>11</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="n">
+        <v>898</v>
+      </c>
+      <c r="S14" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1321,7 +1453,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1353,8 +1485,17 @@
       <c r="P15" t="n">
         <v>13</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="n">
+        <v>966</v>
+      </c>
+      <c r="S15" t="n">
         <v>0</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1382,7 +1523,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1414,8 +1555,17 @@
       <c r="P16" t="n">
         <v>17</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="n">
+        <v>819</v>
+      </c>
+      <c r="S16" t="n">
         <v>0</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1443,7 +1593,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1475,8 +1625,17 @@
       <c r="P17" t="n">
         <v>15</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="n">
+        <v>784</v>
+      </c>
+      <c r="S17" t="n">
         <v>0.01</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1504,7 +1663,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1536,8 +1695,17 @@
       <c r="P18" t="n">
         <v>22</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="n">
+        <v>856</v>
+      </c>
+      <c r="S18" t="n">
         <v>0</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -1565,7 +1733,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1597,8 +1765,21 @@
       <c r="P19" t="n">
         <v>22</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1/4/1 17:00 LMT</t>
+        </is>
+      </c>
+      <c r="R19" t="n">
+        <v>991</v>
+      </c>
+      <c r="S19" t="n">
         <v>0</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1626,7 +1807,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1658,8 +1839,17 @@
       <c r="P20" t="n">
         <v>17</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="n">
+        <v>952</v>
+      </c>
+      <c r="S20" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1687,7 +1877,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1719,8 +1909,17 @@
       <c r="P21" t="n">
         <v>22</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="n">
+        <v>973</v>
+      </c>
+      <c r="S21" t="n">
         <v>0</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -1748,7 +1947,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1780,8 +1979,17 @@
       <c r="P22" t="n">
         <v>16</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="n">
+        <v>966</v>
+      </c>
+      <c r="S22" t="n">
         <v>0</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -1809,7 +2017,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1841,8 +2049,17 @@
       <c r="P23" t="n">
         <v>26</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="n">
+        <v>892</v>
+      </c>
+      <c r="S23" t="n">
         <v>0</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1870,7 +2087,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1902,8 +2119,17 @@
       <c r="P24" t="n">
         <v>13</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="n">
+        <v>771</v>
+      </c>
+      <c r="S24" t="n">
         <v>0</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1931,7 +2157,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1963,8 +2189,17 @@
       <c r="P25" t="n">
         <v>16</v>
       </c>
-      <c r="Q25" t="n">
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="n">
+        <v>968</v>
+      </c>
+      <c r="S25" t="n">
         <v>0.03</v>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1992,7 +2227,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2024,8 +2259,17 @@
       <c r="P26" t="n">
         <v>16</v>
       </c>
-      <c r="Q26" t="n">
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="n">
+        <v>825</v>
+      </c>
+      <c r="S26" t="n">
         <v>0</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -2053,7 +2297,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2085,8 +2329,17 @@
       <c r="P27" t="n">
         <v>17</v>
       </c>
-      <c r="Q27" t="n">
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="n">
+        <v>982</v>
+      </c>
+      <c r="S27" t="n">
         <v>0</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -2114,7 +2367,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2146,8 +2399,17 @@
       <c r="P28" t="n">
         <v>21</v>
       </c>
-      <c r="Q28" t="n">
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="n">
+        <v>939</v>
+      </c>
+      <c r="S28" t="n">
         <v>0</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -2175,7 +2437,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2207,8 +2469,17 @@
       <c r="P29" t="n">
         <v>11</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="n">
+        <v>708</v>
+      </c>
+      <c r="S29" t="n">
         <v>0</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -2236,7 +2507,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2268,8 +2539,17 @@
       <c r="P30" t="n">
         <v>23</v>
       </c>
-      <c r="Q30" t="n">
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="n">
+        <v>886</v>
+      </c>
+      <c r="S30" t="n">
         <v>0</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -2297,7 +2577,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2329,8 +2609,17 @@
       <c r="P31" t="n">
         <v>13</v>
       </c>
-      <c r="Q31" t="n">
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="n">
+        <v>953</v>
+      </c>
+      <c r="S31" t="n">
         <v>0</v>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -2358,7 +2647,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2390,8 +2679,17 @@
       <c r="P32" t="n">
         <v>18</v>
       </c>
-      <c r="Q32" t="n">
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="n">
+        <v>904</v>
+      </c>
+      <c r="S32" t="n">
         <v>0</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -2419,7 +2717,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2451,8 +2749,17 @@
       <c r="P33" t="n">
         <v>17</v>
       </c>
-      <c r="Q33" t="n">
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="n">
+        <v>717</v>
+      </c>
+      <c r="S33" t="n">
         <v>0.08</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -2480,7 +2787,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2512,8 +2819,17 @@
       <c r="P34" t="n">
         <v>13</v>
       </c>
-      <c r="Q34" t="n">
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="n">
+        <v>763</v>
+      </c>
+      <c r="S34" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -2541,7 +2857,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2573,8 +2889,17 @@
       <c r="P35" t="n">
         <v>16</v>
       </c>
-      <c r="Q35" t="n">
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="n">
+        <v>851</v>
+      </c>
+      <c r="S35" t="n">
         <v>0.03</v>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -2602,7 +2927,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2634,8 +2959,17 @@
       <c r="P36" t="n">
         <v>15</v>
       </c>
-      <c r="Q36" t="n">
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="n">
+        <v>728</v>
+      </c>
+      <c r="S36" t="n">
         <v>0.06</v>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -2663,7 +2997,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2695,8 +3029,17 @@
       <c r="P37" t="n">
         <v>19</v>
       </c>
-      <c r="Q37" t="n">
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="n">
+        <v>814</v>
+      </c>
+      <c r="S37" t="n">
         <v>0</v>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -2724,7 +3067,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2756,8 +3099,17 @@
       <c r="P38" t="n">
         <v>24</v>
       </c>
-      <c r="Q38" t="n">
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="n">
+        <v>904</v>
+      </c>
+      <c r="S38" t="n">
         <v>0</v>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -2785,7 +3137,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2817,8 +3169,17 @@
       <c r="P39" t="n">
         <v>21</v>
       </c>
-      <c r="Q39" t="n">
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="n">
+        <v>992</v>
+      </c>
+      <c r="S39" t="n">
         <v>0</v>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -2846,7 +3207,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2878,8 +3239,17 @@
       <c r="P40" t="n">
         <v>15</v>
       </c>
-      <c r="Q40" t="n">
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="n">
+        <v>892</v>
+      </c>
+      <c r="S40" t="n">
         <v>0</v>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -2907,7 +3277,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2939,8 +3309,17 @@
       <c r="P41" t="n">
         <v>16</v>
       </c>
-      <c r="Q41" t="n">
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="n">
+        <v>822</v>
+      </c>
+      <c r="S41" t="n">
         <v>0</v>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -2968,7 +3347,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3000,8 +3379,17 @@
       <c r="P42" t="n">
         <v>17</v>
       </c>
-      <c r="Q42" t="n">
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="n">
+        <v>846</v>
+      </c>
+      <c r="S42" t="n">
         <v>0</v>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -3029,7 +3417,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3061,8 +3449,17 @@
       <c r="P43" t="n">
         <v>19</v>
       </c>
-      <c r="Q43" t="n">
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="n">
+        <v>955</v>
+      </c>
+      <c r="S43" t="n">
         <v>0</v>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -3090,7 +3487,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3122,8 +3519,17 @@
       <c r="P44" t="n">
         <v>18</v>
       </c>
-      <c r="Q44" t="n">
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="n">
+        <v>800</v>
+      </c>
+      <c r="S44" t="n">
         <v>0</v>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -3151,7 +3557,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3183,8 +3589,17 @@
       <c r="P45" t="n">
         <v>21</v>
       </c>
-      <c r="Q45" t="n">
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="n">
+        <v>952</v>
+      </c>
+      <c r="S45" t="n">
         <v>0</v>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -3212,7 +3627,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3244,8 +3659,17 @@
       <c r="P46" t="n">
         <v>16</v>
       </c>
-      <c r="Q46" t="n">
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="n">
+        <v>963</v>
+      </c>
+      <c r="S46" t="n">
         <v>0.03</v>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -3273,7 +3697,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3305,8 +3729,17 @@
       <c r="P47" t="n">
         <v>15</v>
       </c>
-      <c r="Q47" t="n">
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="n">
+        <v>658</v>
+      </c>
+      <c r="S47" t="n">
         <v>0</v>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -3334,7 +3767,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -3366,8 +3799,17 @@
       <c r="P48" t="n">
         <v>22</v>
       </c>
-      <c r="Q48" t="n">
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="n">
+        <v>939</v>
+      </c>
+      <c r="S48" t="n">
         <v>0</v>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -3395,7 +3837,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -3427,8 +3869,17 @@
       <c r="P49" t="n">
         <v>17</v>
       </c>
-      <c r="Q49" t="n">
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="n">
+        <v>688</v>
+      </c>
+      <c r="S49" t="n">
         <v>0</v>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -3456,7 +3907,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -3488,8 +3939,17 @@
       <c r="P50" t="n">
         <v>17</v>
       </c>
-      <c r="Q50" t="n">
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="n">
+        <v>789</v>
+      </c>
+      <c r="S50" t="n">
         <v>0</v>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -3517,7 +3977,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3549,8 +4009,17 @@
       <c r="P51" t="n">
         <v>24</v>
       </c>
-      <c r="Q51" t="n">
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="n">
+        <v>929</v>
+      </c>
+      <c r="S51" t="n">
         <v>0</v>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -3578,7 +4047,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3610,8 +4079,17 @@
       <c r="P52" t="n">
         <v>9</v>
       </c>
-      <c r="Q52" t="n">
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="n">
+        <v>987</v>
+      </c>
+      <c r="S52" t="n">
         <v>0.01</v>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -3639,7 +4117,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3671,8 +4149,17 @@
       <c r="P53" t="n">
         <v>17</v>
       </c>
-      <c r="Q53" t="n">
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="n">
+        <v>940</v>
+      </c>
+      <c r="S53" t="n">
         <v>0</v>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -3700,7 +4187,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3732,8 +4219,17 @@
       <c r="P54" t="n">
         <v>24</v>
       </c>
-      <c r="Q54" t="n">
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="n">
+        <v>743</v>
+      </c>
+      <c r="S54" t="n">
         <v>0</v>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -3761,7 +4257,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3793,8 +4289,17 @@
       <c r="P55" t="n">
         <v>16</v>
       </c>
-      <c r="Q55" t="n">
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="n">
+        <v>899</v>
+      </c>
+      <c r="S55" t="n">
         <v>0</v>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -3822,7 +4327,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3854,8 +4359,17 @@
       <c r="P56" t="n">
         <v>13</v>
       </c>
-      <c r="Q56" t="n">
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="n">
+        <v>865</v>
+      </c>
+      <c r="S56" t="n">
         <v>0</v>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -3883,7 +4397,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -3915,8 +4429,17 @@
       <c r="P57" t="n">
         <v>17</v>
       </c>
-      <c r="Q57" t="n">
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="n">
+        <v>686</v>
+      </c>
+      <c r="S57" t="n">
         <v>0</v>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -3944,7 +4467,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3976,8 +4499,17 @@
       <c r="P58" t="n">
         <v>11</v>
       </c>
-      <c r="Q58" t="n">
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="n">
+        <v>656</v>
+      </c>
+      <c r="S58" t="n">
         <v>0.05</v>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -4005,7 +4537,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4037,8 +4569,17 @@
       <c r="P59" t="n">
         <v>22</v>
       </c>
-      <c r="Q59" t="n">
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="n">
+        <v>910</v>
+      </c>
+      <c r="S59" t="n">
         <v>0</v>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -4066,7 +4607,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -4098,8 +4639,17 @@
       <c r="P60" t="n">
         <v>24</v>
       </c>
-      <c r="Q60" t="n">
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="n">
+        <v>978</v>
+      </c>
+      <c r="S60" t="n">
         <v>0</v>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -4127,7 +4677,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -4159,8 +4709,17 @@
       <c r="P61" t="n">
         <v>14</v>
       </c>
-      <c r="Q61" t="n">
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="n">
+        <v>996</v>
+      </c>
+      <c r="S61" t="n">
         <v>0</v>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -4188,7 +4747,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -4220,8 +4779,17 @@
       <c r="P62" t="n">
         <v>17</v>
       </c>
-      <c r="Q62" t="n">
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="n">
+        <v>693</v>
+      </c>
+      <c r="S62" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -4249,7 +4817,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -4281,8 +4849,17 @@
       <c r="P63" t="n">
         <v>21</v>
       </c>
-      <c r="Q63" t="n">
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="n">
+        <v>892</v>
+      </c>
+      <c r="S63" t="n">
         <v>0</v>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -4310,7 +4887,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -4342,8 +4919,17 @@
       <c r="P64" t="n">
         <v>13</v>
       </c>
-      <c r="Q64" t="n">
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="n">
+        <v>996</v>
+      </c>
+      <c r="S64" t="n">
         <v>0</v>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -4371,7 +4957,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -4403,8 +4989,17 @@
       <c r="P65" t="n">
         <v>15</v>
       </c>
-      <c r="Q65" t="n">
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="n">
+        <v>716</v>
+      </c>
+      <c r="S65" t="n">
         <v>0.03</v>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -4432,7 +5027,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -4464,8 +5059,17 @@
       <c r="P66" t="n">
         <v>18</v>
       </c>
-      <c r="Q66" t="n">
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="n">
+        <v>955</v>
+      </c>
+      <c r="S66" t="n">
         <v>0</v>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -4493,7 +5097,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -4525,8 +5129,17 @@
       <c r="P67" t="n">
         <v>24</v>
       </c>
-      <c r="Q67" t="n">
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="n">
+        <v>839</v>
+      </c>
+      <c r="S67" t="n">
         <v>0</v>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -4554,7 +5167,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -4586,8 +5199,17 @@
       <c r="P68" t="n">
         <v>14</v>
       </c>
-      <c r="Q68" t="n">
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="n">
+        <v>930</v>
+      </c>
+      <c r="S68" t="n">
         <v>0.11</v>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -4615,7 +5237,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -4647,8 +5269,17 @@
       <c r="P69" t="n">
         <v>21</v>
       </c>
-      <c r="Q69" t="n">
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="n">
+        <v>965</v>
+      </c>
+      <c r="S69" t="n">
         <v>0.01</v>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -4676,7 +5307,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -4708,8 +5339,17 @@
       <c r="P70" t="n">
         <v>23</v>
       </c>
-      <c r="Q70" t="n">
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="n">
+        <v>858</v>
+      </c>
+      <c r="S70" t="n">
         <v>0.04</v>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -4737,7 +5377,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -4769,8 +5409,17 @@
       <c r="P71" t="n">
         <v>25</v>
       </c>
-      <c r="Q71" t="n">
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="n">
+        <v>930</v>
+      </c>
+      <c r="S71" t="n">
         <v>0</v>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -4798,7 +5447,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -4830,8 +5479,17 @@
       <c r="P72" t="n">
         <v>16</v>
       </c>
-      <c r="Q72" t="n">
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="n">
+        <v>764</v>
+      </c>
+      <c r="S72" t="n">
         <v>0.04</v>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -4859,7 +5517,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -4891,8 +5549,17 @@
       <c r="P73" t="n">
         <v>17</v>
       </c>
-      <c r="Q73" t="n">
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="n">
+        <v>675</v>
+      </c>
+      <c r="S73" t="n">
         <v>0.03</v>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -4920,7 +5587,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -4952,8 +5619,17 @@
       <c r="P74" t="n">
         <v>16</v>
       </c>
-      <c r="Q74" t="n">
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="n">
+        <v>808</v>
+      </c>
+      <c r="S74" t="n">
         <v>0.01</v>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -4981,7 +5657,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -5013,8 +5689,17 @@
       <c r="P75" t="n">
         <v>16</v>
       </c>
-      <c r="Q75" t="n">
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="n">
+        <v>898</v>
+      </c>
+      <c r="S75" t="n">
         <v>0</v>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -5042,7 +5727,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -5074,8 +5759,17 @@
       <c r="P76" t="n">
         <v>11</v>
       </c>
-      <c r="Q76" t="n">
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="n">
+        <v>710</v>
+      </c>
+      <c r="S76" t="n">
         <v>0.03</v>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -5103,7 +5797,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -5135,8 +5829,17 @@
       <c r="P77" t="n">
         <v>13</v>
       </c>
-      <c r="Q77" t="n">
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="n">
+        <v>906</v>
+      </c>
+      <c r="S77" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -5164,7 +5867,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -5196,8 +5899,17 @@
       <c r="P78" t="n">
         <v>15</v>
       </c>
-      <c r="Q78" t="n">
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="n">
+        <v>871</v>
+      </c>
+      <c r="S78" t="n">
         <v>0</v>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -5225,7 +5937,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -5257,8 +5969,17 @@
       <c r="P79" t="n">
         <v>16</v>
       </c>
-      <c r="Q79" t="n">
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="n">
+        <v>818</v>
+      </c>
+      <c r="S79" t="n">
         <v>0</v>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -5286,7 +6007,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -5318,8 +6039,17 @@
       <c r="P80" t="n">
         <v>11</v>
       </c>
-      <c r="Q80" t="n">
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="n">
+        <v>916</v>
+      </c>
+      <c r="S80" t="n">
         <v>0</v>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -5347,7 +6077,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -5379,8 +6109,17 @@
       <c r="P81" t="n">
         <v>17</v>
       </c>
-      <c r="Q81" t="n">
+      <c r="Q81" t="inlineStr"/>
+      <c r="R81" t="n">
+        <v>910</v>
+      </c>
+      <c r="S81" t="n">
         <v>0</v>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -5408,7 +6147,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -5440,8 +6179,17 @@
       <c r="P82" t="n">
         <v>16</v>
       </c>
-      <c r="Q82" t="n">
+      <c r="Q82" t="inlineStr"/>
+      <c r="R82" t="n">
+        <v>922</v>
+      </c>
+      <c r="S82" t="n">
         <v>0</v>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -5469,7 +6217,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -5501,8 +6249,17 @@
       <c r="P83" t="n">
         <v>14</v>
       </c>
-      <c r="Q83" t="n">
+      <c r="Q83" t="inlineStr"/>
+      <c r="R83" t="n">
+        <v>978</v>
+      </c>
+      <c r="S83" t="n">
         <v>0</v>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -5530,7 +6287,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -5562,8 +6319,17 @@
       <c r="P84" t="n">
         <v>19</v>
       </c>
-      <c r="Q84" t="n">
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="n">
+        <v>901</v>
+      </c>
+      <c r="S84" t="n">
         <v>0</v>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -5591,7 +6357,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -5623,8 +6389,17 @@
       <c r="P85" t="n">
         <v>14</v>
       </c>
-      <c r="Q85" t="n">
+      <c r="Q85" t="inlineStr"/>
+      <c r="R85" t="n">
+        <v>929</v>
+      </c>
+      <c r="S85" t="n">
         <v>0</v>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -5652,7 +6427,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -5684,8 +6459,17 @@
       <c r="P86" t="n">
         <v>13</v>
       </c>
-      <c r="Q86" t="n">
+      <c r="Q86" t="inlineStr"/>
+      <c r="R86" t="n">
+        <v>740</v>
+      </c>
+      <c r="S86" t="n">
         <v>0</v>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -5713,7 +6497,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -5745,8 +6529,17 @@
       <c r="P87" t="n">
         <v>19</v>
       </c>
-      <c r="Q87" t="n">
+      <c r="Q87" t="inlineStr"/>
+      <c r="R87" t="n">
+        <v>853</v>
+      </c>
+      <c r="S87" t="n">
         <v>0.01</v>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="88">
@@ -5774,7 +6567,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -5806,8 +6599,17 @@
       <c r="P88" t="n">
         <v>13</v>
       </c>
-      <c r="Q88" t="n">
+      <c r="Q88" t="inlineStr"/>
+      <c r="R88" t="n">
+        <v>815</v>
+      </c>
+      <c r="S88" t="n">
         <v>0</v>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -5835,7 +6637,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -5867,8 +6669,17 @@
       <c r="P89" t="n">
         <v>24</v>
       </c>
-      <c r="Q89" t="n">
+      <c r="Q89" t="inlineStr"/>
+      <c r="R89" t="n">
+        <v>906</v>
+      </c>
+      <c r="S89" t="n">
         <v>0</v>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -5896,7 +6707,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -5928,8 +6739,17 @@
       <c r="P90" t="n">
         <v>14</v>
       </c>
-      <c r="Q90" t="n">
+      <c r="Q90" t="inlineStr"/>
+      <c r="R90" t="n">
+        <v>624</v>
+      </c>
+      <c r="S90" t="n">
         <v>0.03</v>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -5957,7 +6777,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -5989,8 +6809,17 @@
       <c r="P91" t="n">
         <v>17</v>
       </c>
-      <c r="Q91" t="n">
+      <c r="Q91" t="inlineStr"/>
+      <c r="R91" t="n">
+        <v>809</v>
+      </c>
+      <c r="S91" t="n">
         <v>0.01</v>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="92">
@@ -6018,7 +6847,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -6050,8 +6879,17 @@
       <c r="P92" t="n">
         <v>16</v>
       </c>
-      <c r="Q92" t="n">
+      <c r="Q92" t="inlineStr"/>
+      <c r="R92" t="n">
+        <v>976</v>
+      </c>
+      <c r="S92" t="n">
         <v>0</v>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -6079,7 +6917,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -6111,8 +6949,17 @@
       <c r="P93" t="n">
         <v>10</v>
       </c>
-      <c r="Q93" t="n">
+      <c r="Q93" t="inlineStr"/>
+      <c r="R93" t="n">
+        <v>715</v>
+      </c>
+      <c r="S93" t="n">
         <v>0</v>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -6140,7 +6987,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -6172,8 +7019,17 @@
       <c r="P94" t="n">
         <v>24</v>
       </c>
-      <c r="Q94" t="n">
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="n">
+        <v>915</v>
+      </c>
+      <c r="S94" t="n">
         <v>0</v>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -6201,7 +7057,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -6233,8 +7089,17 @@
       <c r="P95" t="n">
         <v>17</v>
       </c>
-      <c r="Q95" t="n">
+      <c r="Q95" t="inlineStr"/>
+      <c r="R95" t="n">
+        <v>978</v>
+      </c>
+      <c r="S95" t="n">
         <v>0</v>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -6262,7 +7127,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -6294,8 +7159,17 @@
       <c r="P96" t="n">
         <v>24</v>
       </c>
-      <c r="Q96" t="n">
+      <c r="Q96" t="inlineStr"/>
+      <c r="R96" t="n">
+        <v>733</v>
+      </c>
+      <c r="S96" t="n">
         <v>0</v>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -6323,7 +7197,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -6355,8 +7229,17 @@
       <c r="P97" t="n">
         <v>15</v>
       </c>
-      <c r="Q97" t="n">
+      <c r="Q97" t="inlineStr"/>
+      <c r="R97" t="n">
+        <v>724</v>
+      </c>
+      <c r="S97" t="n">
         <v>0</v>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="98">
@@ -6384,7 +7267,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -6416,8 +7299,17 @@
       <c r="P98" t="n">
         <v>16</v>
       </c>
-      <c r="Q98" t="n">
+      <c r="Q98" t="inlineStr"/>
+      <c r="R98" t="n">
+        <v>916</v>
+      </c>
+      <c r="S98" t="n">
         <v>0</v>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -6445,7 +7337,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -6477,8 +7369,17 @@
       <c r="P99" t="n">
         <v>19</v>
       </c>
-      <c r="Q99" t="n">
+      <c r="Q99" t="inlineStr"/>
+      <c r="R99" t="n">
+        <v>903</v>
+      </c>
+      <c r="S99" t="n">
         <v>0</v>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -6506,7 +7407,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -6538,8 +7439,17 @@
       <c r="P100" t="n">
         <v>15</v>
       </c>
-      <c r="Q100" t="n">
+      <c r="Q100" t="inlineStr"/>
+      <c r="R100" t="n">
+        <v>982</v>
+      </c>
+      <c r="S100" t="n">
         <v>0</v>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -6567,7 +7477,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -6599,8 +7509,17 @@
       <c r="P101" t="n">
         <v>14</v>
       </c>
-      <c r="Q101" t="n">
+      <c r="Q101" t="inlineStr"/>
+      <c r="R101" t="n">
+        <v>791</v>
+      </c>
+      <c r="S101" t="n">
         <v>0</v>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -6628,7 +7547,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -6660,8 +7579,17 @@
       <c r="P102" t="n">
         <v>15</v>
       </c>
-      <c r="Q102" t="n">
+      <c r="Q102" t="inlineStr"/>
+      <c r="R102" t="n">
+        <v>969</v>
+      </c>
+      <c r="S102" t="n">
         <v>0</v>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -6689,7 +7617,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -6721,8 +7649,17 @@
       <c r="P103" t="n">
         <v>25</v>
       </c>
-      <c r="Q103" t="n">
+      <c r="Q103" t="inlineStr"/>
+      <c r="R103" t="n">
+        <v>902</v>
+      </c>
+      <c r="S103" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="104">
@@ -6750,7 +7687,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -6782,8 +7719,17 @@
       <c r="P104" t="n">
         <v>24</v>
       </c>
-      <c r="Q104" t="n">
+      <c r="Q104" t="inlineStr"/>
+      <c r="R104" t="n">
+        <v>934</v>
+      </c>
+      <c r="S104" t="n">
         <v>0</v>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -6811,7 +7757,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -6843,8 +7789,17 @@
       <c r="P105" t="n">
         <v>23</v>
       </c>
-      <c r="Q105" t="n">
+      <c r="Q105" t="inlineStr"/>
+      <c r="R105" t="n">
+        <v>962</v>
+      </c>
+      <c r="S105" t="n">
         <v>0</v>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -6872,7 +7827,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -6904,8 +7859,17 @@
       <c r="P106" t="n">
         <v>16</v>
       </c>
-      <c r="Q106" t="n">
+      <c r="Q106" t="inlineStr"/>
+      <c r="R106" t="n">
+        <v>805</v>
+      </c>
+      <c r="S106" t="n">
         <v>0</v>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="107">
@@ -6933,7 +7897,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -6965,8 +7929,17 @@
       <c r="P107" t="n">
         <v>14</v>
       </c>
-      <c r="Q107" t="n">
+      <c r="Q107" t="inlineStr"/>
+      <c r="R107" t="n">
+        <v>870</v>
+      </c>
+      <c r="S107" t="n">
         <v>0</v>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="108">
@@ -6994,7 +7967,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -7026,8 +7999,17 @@
       <c r="P108" t="n">
         <v>21</v>
       </c>
-      <c r="Q108" t="n">
+      <c r="Q108" t="inlineStr"/>
+      <c r="R108" t="n">
+        <v>948</v>
+      </c>
+      <c r="S108" t="n">
         <v>0.04</v>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -7055,7 +8037,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -7087,8 +8069,17 @@
       <c r="P109" t="n">
         <v>13</v>
       </c>
-      <c r="Q109" t="n">
+      <c r="Q109" t="inlineStr"/>
+      <c r="R109" t="n">
+        <v>916</v>
+      </c>
+      <c r="S109" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="110">
@@ -7116,7 +8107,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -7148,8 +8139,17 @@
       <c r="P110" t="n">
         <v>13</v>
       </c>
-      <c r="Q110" t="n">
+      <c r="Q110" t="inlineStr"/>
+      <c r="R110" t="n">
+        <v>918</v>
+      </c>
+      <c r="S110" t="n">
         <v>0</v>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="111">
@@ -7177,7 +8177,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -7209,8 +8209,17 @@
       <c r="P111" t="n">
         <v>14</v>
       </c>
-      <c r="Q111" t="n">
+      <c r="Q111" t="inlineStr"/>
+      <c r="R111" t="n">
+        <v>800</v>
+      </c>
+      <c r="S111" t="n">
         <v>0</v>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="112">
@@ -7238,7 +8247,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -7270,8 +8279,17 @@
       <c r="P112" t="n">
         <v>14</v>
       </c>
-      <c r="Q112" t="n">
+      <c r="Q112" t="inlineStr"/>
+      <c r="R112" t="n">
+        <v>866</v>
+      </c>
+      <c r="S112" t="n">
         <v>0.04</v>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="113">
@@ -7299,7 +8317,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -7331,8 +8349,17 @@
       <c r="P113" t="n">
         <v>13</v>
       </c>
-      <c r="Q113" t="n">
+      <c r="Q113" t="inlineStr"/>
+      <c r="R113" t="n">
+        <v>756</v>
+      </c>
+      <c r="S113" t="n">
         <v>0.04</v>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="114">
@@ -7360,7 +8387,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -7392,8 +8419,17 @@
       <c r="P114" t="n">
         <v>13</v>
       </c>
-      <c r="Q114" t="n">
+      <c r="Q114" t="inlineStr"/>
+      <c r="R114" t="n">
+        <v>890</v>
+      </c>
+      <c r="S114" t="n">
         <v>0</v>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="115">
@@ -7421,7 +8457,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -7453,8 +8489,17 @@
       <c r="P115" t="n">
         <v>11</v>
       </c>
-      <c r="Q115" t="n">
+      <c r="Q115" t="inlineStr"/>
+      <c r="R115" t="n">
+        <v>813</v>
+      </c>
+      <c r="S115" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="116">
@@ -7482,7 +8527,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -7514,8 +8559,17 @@
       <c r="P116" t="n">
         <v>18</v>
       </c>
-      <c r="Q116" t="n">
+      <c r="Q116" t="inlineStr"/>
+      <c r="R116" t="n">
+        <v>968</v>
+      </c>
+      <c r="S116" t="n">
         <v>0</v>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="117">
@@ -7543,7 +8597,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -7575,8 +8629,17 @@
       <c r="P117" t="n">
         <v>19</v>
       </c>
-      <c r="Q117" t="n">
+      <c r="Q117" t="inlineStr"/>
+      <c r="R117" t="n">
+        <v>906</v>
+      </c>
+      <c r="S117" t="n">
         <v>0</v>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="118">
@@ -7604,7 +8667,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -7636,8 +8699,17 @@
       <c r="P118" t="n">
         <v>15</v>
       </c>
-      <c r="Q118" t="n">
+      <c r="Q118" t="inlineStr"/>
+      <c r="R118" t="n">
+        <v>979</v>
+      </c>
+      <c r="S118" t="n">
         <v>0</v>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="119">
@@ -7665,7 +8737,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -7697,8 +8769,17 @@
       <c r="P119" t="n">
         <v>8</v>
       </c>
-      <c r="Q119" t="n">
+      <c r="Q119" t="inlineStr"/>
+      <c r="R119" t="n">
+        <v>827</v>
+      </c>
+      <c r="S119" t="n">
         <v>0</v>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -7726,7 +8807,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -7758,8 +8839,17 @@
       <c r="P120" t="n">
         <v>17</v>
       </c>
-      <c r="Q120" t="n">
+      <c r="Q120" t="inlineStr"/>
+      <c r="R120" t="n">
+        <v>836</v>
+      </c>
+      <c r="S120" t="n">
         <v>0.01</v>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="121">
@@ -7787,7 +8877,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -7819,8 +8909,17 @@
       <c r="P121" t="n">
         <v>14</v>
       </c>
-      <c r="Q121" t="n">
+      <c r="Q121" t="inlineStr"/>
+      <c r="R121" t="n">
+        <v>924</v>
+      </c>
+      <c r="S121" t="n">
         <v>0</v>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="122">
@@ -7848,7 +8947,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -7880,8 +8979,17 @@
       <c r="P122" t="n">
         <v>15</v>
       </c>
-      <c r="Q122" t="n">
+      <c r="Q122" t="inlineStr"/>
+      <c r="R122" t="n">
+        <v>997</v>
+      </c>
+      <c r="S122" t="n">
         <v>0</v>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="123">
@@ -7909,7 +9017,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -7941,8 +9049,17 @@
       <c r="P123" t="n">
         <v>15</v>
       </c>
-      <c r="Q123" t="n">
+      <c r="Q123" t="inlineStr"/>
+      <c r="R123" t="n">
+        <v>942</v>
+      </c>
+      <c r="S123" t="n">
         <v>0</v>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -7970,7 +9087,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -8002,8 +9119,17 @@
       <c r="P124" t="n">
         <v>16</v>
       </c>
-      <c r="Q124" t="n">
+      <c r="Q124" t="inlineStr"/>
+      <c r="R124" t="n">
+        <v>990</v>
+      </c>
+      <c r="S124" t="n">
         <v>0</v>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="125">
@@ -8031,7 +9157,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -8063,8 +9189,17 @@
       <c r="P125" t="n">
         <v>23</v>
       </c>
-      <c r="Q125" t="n">
+      <c r="Q125" t="inlineStr"/>
+      <c r="R125" t="n">
+        <v>958</v>
+      </c>
+      <c r="S125" t="n">
         <v>0</v>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="126">
@@ -8092,7 +9227,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -8124,8 +9259,17 @@
       <c r="P126" t="n">
         <v>16</v>
       </c>
-      <c r="Q126" t="n">
+      <c r="Q126" t="inlineStr"/>
+      <c r="R126" t="n">
+        <v>966</v>
+      </c>
+      <c r="S126" t="n">
         <v>0</v>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="127">
@@ -8153,7 +9297,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -8185,8 +9329,17 @@
       <c r="P127" t="n">
         <v>15</v>
       </c>
-      <c r="Q127" t="n">
+      <c r="Q127" t="inlineStr"/>
+      <c r="R127" t="n">
+        <v>955</v>
+      </c>
+      <c r="S127" t="n">
         <v>0</v>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="128">
@@ -8214,7 +9367,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -8246,8 +9399,17 @@
       <c r="P128" t="n">
         <v>17</v>
       </c>
-      <c r="Q128" t="n">
+      <c r="Q128" t="inlineStr"/>
+      <c r="R128" t="n">
+        <v>894</v>
+      </c>
+      <c r="S128" t="n">
         <v>0</v>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="129">
@@ -8275,7 +9437,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -8307,8 +9469,17 @@
       <c r="P129" t="n">
         <v>17</v>
       </c>
-      <c r="Q129" t="n">
+      <c r="Q129" t="inlineStr"/>
+      <c r="R129" t="n">
+        <v>918</v>
+      </c>
+      <c r="S129" t="n">
         <v>0.03</v>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="130">
@@ -8336,7 +9507,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -8368,8 +9539,17 @@
       <c r="P130" t="n">
         <v>15</v>
       </c>
-      <c r="Q130" t="n">
+      <c r="Q130" t="inlineStr"/>
+      <c r="R130" t="n">
+        <v>960</v>
+      </c>
+      <c r="S130" t="n">
         <v>0.04</v>
+      </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="131">
@@ -8397,7 +9577,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -8429,8 +9609,17 @@
       <c r="P131" t="n">
         <v>17</v>
       </c>
-      <c r="Q131" t="n">
+      <c r="Q131" t="inlineStr"/>
+      <c r="R131" t="n">
+        <v>908</v>
+      </c>
+      <c r="S131" t="n">
         <v>0</v>
+      </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="132">
@@ -8458,7 +9647,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -8490,8 +9679,17 @@
       <c r="P132" t="n">
         <v>15</v>
       </c>
-      <c r="Q132" t="n">
+      <c r="Q132" t="inlineStr"/>
+      <c r="R132" t="n">
+        <v>969</v>
+      </c>
+      <c r="S132" t="n">
         <v>0</v>
+      </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="133">
@@ -8519,7 +9717,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -8551,8 +9749,17 @@
       <c r="P133" t="n">
         <v>14</v>
       </c>
-      <c r="Q133" t="n">
+      <c r="Q133" t="inlineStr"/>
+      <c r="R133" t="n">
+        <v>812</v>
+      </c>
+      <c r="S133" t="n">
         <v>0</v>
+      </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="134">
@@ -8580,7 +9787,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -8612,8 +9819,17 @@
       <c r="P134" t="n">
         <v>19</v>
       </c>
-      <c r="Q134" t="n">
+      <c r="Q134" t="inlineStr"/>
+      <c r="R134" t="n">
+        <v>705</v>
+      </c>
+      <c r="S134" t="n">
         <v>0</v>
+      </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="135">
@@ -8641,7 +9857,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -8673,8 +9889,17 @@
       <c r="P135" t="n">
         <v>18</v>
       </c>
-      <c r="Q135" t="n">
+      <c r="Q135" t="inlineStr"/>
+      <c r="R135" t="n">
+        <v>931</v>
+      </c>
+      <c r="S135" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="136">
@@ -8702,7 +9927,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -8734,8 +9959,17 @@
       <c r="P136" t="n">
         <v>15</v>
       </c>
-      <c r="Q136" t="n">
+      <c r="Q136" t="inlineStr"/>
+      <c r="R136" t="n">
+        <v>744</v>
+      </c>
+      <c r="S136" t="n">
         <v>0</v>
+      </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="137">
@@ -8763,7 +9997,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -8795,8 +10029,17 @@
       <c r="P137" t="n">
         <v>15</v>
       </c>
-      <c r="Q137" t="n">
+      <c r="Q137" t="inlineStr"/>
+      <c r="R137" t="n">
+        <v>881</v>
+      </c>
+      <c r="S137" t="n">
         <v>0</v>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="138">
@@ -8824,7 +10067,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -8856,8 +10099,17 @@
       <c r="P138" t="n">
         <v>22</v>
       </c>
-      <c r="Q138" t="n">
+      <c r="Q138" t="inlineStr"/>
+      <c r="R138" t="n">
+        <v>934</v>
+      </c>
+      <c r="S138" t="n">
         <v>0</v>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="139">
@@ -8885,7 +10137,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -8917,8 +10169,17 @@
       <c r="P139" t="n">
         <v>19</v>
       </c>
-      <c r="Q139" t="n">
+      <c r="Q139" t="inlineStr"/>
+      <c r="R139" t="n">
+        <v>871</v>
+      </c>
+      <c r="S139" t="n">
         <v>0</v>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="140">
@@ -8946,7 +10207,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -8978,8 +10239,17 @@
       <c r="P140" t="n">
         <v>16</v>
       </c>
-      <c r="Q140" t="n">
+      <c r="Q140" t="inlineStr"/>
+      <c r="R140" t="n">
+        <v>917</v>
+      </c>
+      <c r="S140" t="n">
         <v>0.03</v>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="141">
@@ -9007,7 +10277,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -9039,8 +10309,17 @@
       <c r="P141" t="n">
         <v>19</v>
       </c>
-      <c r="Q141" t="n">
+      <c r="Q141" t="inlineStr"/>
+      <c r="R141" t="n">
+        <v>872</v>
+      </c>
+      <c r="S141" t="n">
         <v>0.02</v>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="142">
@@ -9068,7 +10347,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -9100,8 +10379,17 @@
       <c r="P142" t="n">
         <v>19</v>
       </c>
-      <c r="Q142" t="n">
+      <c r="Q142" t="inlineStr"/>
+      <c r="R142" t="n">
+        <v>916</v>
+      </c>
+      <c r="S142" t="n">
         <v>0</v>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="143">
@@ -9129,7 +10417,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -9161,8 +10449,17 @@
       <c r="P143" t="n">
         <v>19</v>
       </c>
-      <c r="Q143" t="n">
+      <c r="Q143" t="inlineStr"/>
+      <c r="R143" t="n">
+        <v>819</v>
+      </c>
+      <c r="S143" t="n">
         <v>0.06</v>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="144">
@@ -9190,7 +10487,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -9222,8 +10519,17 @@
       <c r="P144" t="n">
         <v>15</v>
       </c>
-      <c r="Q144" t="n">
+      <c r="Q144" t="inlineStr"/>
+      <c r="R144" t="n">
+        <v>872</v>
+      </c>
+      <c r="S144" t="n">
         <v>0.01</v>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="145">
@@ -9251,7 +10557,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -9283,8 +10589,17 @@
       <c r="P145" t="n">
         <v>23</v>
       </c>
-      <c r="Q145" t="n">
+      <c r="Q145" t="inlineStr"/>
+      <c r="R145" t="n">
+        <v>883</v>
+      </c>
+      <c r="S145" t="n">
         <v>0.04</v>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="146">
@@ -9312,7 +10627,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -9344,8 +10659,17 @@
       <c r="P146" t="n">
         <v>15</v>
       </c>
-      <c r="Q146" t="n">
+      <c r="Q146" t="inlineStr"/>
+      <c r="R146" t="n">
+        <v>886</v>
+      </c>
+      <c r="S146" t="n">
         <v>0.14</v>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="147">
@@ -9373,7 +10697,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -9405,8 +10729,21 @@
       <c r="P147" t="n">
         <v>15</v>
       </c>
-      <c r="Q147" t="n">
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>1/6/1 17:00 LMT</t>
+        </is>
+      </c>
+      <c r="R147" t="n">
+        <v>975</v>
+      </c>
+      <c r="S147" t="n">
         <v>0</v>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="148">
@@ -9434,7 +10771,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -9466,8 +10803,17 @@
       <c r="P148" t="n">
         <v>16</v>
       </c>
-      <c r="Q148" t="n">
+      <c r="Q148" t="inlineStr"/>
+      <c r="R148" t="n">
+        <v>887</v>
+      </c>
+      <c r="S148" t="n">
         <v>0.01</v>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="149">
@@ -9495,7 +10841,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -9527,8 +10873,17 @@
       <c r="P149" t="n">
         <v>24</v>
       </c>
-      <c r="Q149" t="n">
+      <c r="Q149" t="inlineStr"/>
+      <c r="R149" t="n">
+        <v>804</v>
+      </c>
+      <c r="S149" t="n">
         <v>0</v>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="150">
@@ -9556,7 +10911,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -9588,8 +10943,17 @@
       <c r="P150" t="n">
         <v>11</v>
       </c>
-      <c r="Q150" t="n">
+      <c r="Q150" t="inlineStr"/>
+      <c r="R150" t="n">
+        <v>829</v>
+      </c>
+      <c r="S150" t="n">
         <v>0</v>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="151">
@@ -9617,7 +10981,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -9649,8 +11013,17 @@
       <c r="P151" t="n">
         <v>31</v>
       </c>
-      <c r="Q151" t="n">
+      <c r="Q151" t="inlineStr"/>
+      <c r="R151" t="n">
+        <v>939</v>
+      </c>
+      <c r="S151" t="n">
         <v>0</v>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="152">
@@ -9678,7 +11051,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -9710,8 +11083,17 @@
       <c r="P152" t="n">
         <v>23</v>
       </c>
-      <c r="Q152" t="n">
+      <c r="Q152" t="inlineStr"/>
+      <c r="R152" t="n">
+        <v>884</v>
+      </c>
+      <c r="S152" t="n">
         <v>0</v>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="153">
@@ -9739,7 +11121,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -9771,8 +11153,17 @@
       <c r="P153" t="n">
         <v>13</v>
       </c>
-      <c r="Q153" t="n">
+      <c r="Q153" t="inlineStr"/>
+      <c r="R153" t="n">
+        <v>744</v>
+      </c>
+      <c r="S153" t="n">
         <v>0.04</v>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="154">
@@ -9800,7 +11191,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -9832,8 +11223,17 @@
       <c r="P154" t="n">
         <v>17</v>
       </c>
-      <c r="Q154" t="n">
+      <c r="Q154" t="inlineStr"/>
+      <c r="R154" t="n">
+        <v>735</v>
+      </c>
+      <c r="S154" t="n">
         <v>0</v>
+      </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="155">
@@ -9861,7 +11261,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -9893,8 +11293,17 @@
       <c r="P155" t="n">
         <v>15</v>
       </c>
-      <c r="Q155" t="n">
+      <c r="Q155" t="inlineStr"/>
+      <c r="R155" t="n">
+        <v>775</v>
+      </c>
+      <c r="S155" t="n">
         <v>0.05</v>
+      </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="156">
@@ -9922,7 +11331,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -9954,8 +11363,17 @@
       <c r="P156" t="n">
         <v>17</v>
       </c>
-      <c r="Q156" t="n">
+      <c r="Q156" t="inlineStr"/>
+      <c r="R156" t="n">
+        <v>716</v>
+      </c>
+      <c r="S156" t="n">
         <v>0.07000000000000001</v>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="157">
@@ -9983,7 +11401,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -10015,8 +11433,17 @@
       <c r="P157" t="n">
         <v>18</v>
       </c>
-      <c r="Q157" t="n">
+      <c r="Q157" t="inlineStr"/>
+      <c r="R157" t="n">
+        <v>880</v>
+      </c>
+      <c r="S157" t="n">
         <v>0</v>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
     <row r="158">
@@ -10044,7 +11471,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>8/22/2026</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -10076,8 +11503,17 @@
       <c r="P158" t="n">
         <v>19</v>
       </c>
-      <c r="Q158" t="n">
+      <c r="Q158" t="inlineStr"/>
+      <c r="R158" t="n">
+        <v>882</v>
+      </c>
+      <c r="S158" t="n">
         <v>0</v>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>